<commit_message>
Error tiempo negativo arreglado
</commit_message>
<xml_diff>
--- a/datosIntentosPValues.xlsx
+++ b/datosIntentosPValues.xlsx
@@ -530,55 +530,55 @@
         <v>0</v>
       </c>
       <c r="C2" t="n">
-        <v>2.860148248845242e-09</v>
+        <v>3.951521354449647e-09</v>
       </c>
       <c r="D2" t="n">
-        <v>0.005778123050014108</v>
+        <v>0.006773669736774259</v>
       </c>
       <c r="E2" t="n">
-        <v>0.5782882316827663</v>
+        <v>0.08654873591454997</v>
       </c>
       <c r="F2" t="n">
-        <v>0.000937594313159404</v>
+        <v>0.0008556422323483821</v>
       </c>
       <c r="G2" t="n">
-        <v>6.369010827378881e-10</v>
+        <v>4.827751365533865e-10</v>
       </c>
       <c r="H2" t="n">
-        <v>4.335244092533622e-10</v>
+        <v>3.290047200228263e-10</v>
       </c>
       <c r="I2" t="n">
-        <v>0.01481162278016307</v>
+        <v>0.0141170298716032</v>
       </c>
       <c r="J2" t="n">
-        <v>1.859067479702329e-11</v>
+        <v>1.324049210776918e-11</v>
       </c>
       <c r="K2" t="n">
-        <v>7.823545746664761e-11</v>
+        <v>5.65297713021527e-11</v>
       </c>
       <c r="L2" t="n">
-        <v>0.09315870253868073</v>
+        <v>0.09178553979175272</v>
       </c>
       <c r="M2" t="n">
-        <v>2.03499470752718e-06</v>
+        <v>1.74318497422886e-06</v>
       </c>
       <c r="N2" t="n">
-        <v>3.437593850426097e-06</v>
+        <v>3.003624054421726e-06</v>
       </c>
       <c r="O2" t="n">
-        <v>0.04057990178849622</v>
+        <v>0.03900395999926402</v>
       </c>
       <c r="P2" t="n">
-        <v>4.407385311917058e-11</v>
+        <v>2.582053559427021e-11</v>
       </c>
       <c r="Q2" t="n">
-        <v>3.71175767927445e-10</v>
+        <v>2.543843960175141e-10</v>
       </c>
       <c r="R2" t="n">
-        <v>0.6702671245435687</v>
+        <v>0.6623627930669869</v>
       </c>
       <c r="S2" t="n">
-        <v>0.5169353273419229</v>
+        <v>0.5098068507681475</v>
       </c>
     </row>
     <row r="3">
@@ -588,58 +588,58 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>2.860148248845242e-09</v>
+        <v>3.951521354449647e-09</v>
       </c>
       <c r="C3" t="n">
         <v>0</v>
       </c>
       <c r="D3" t="n">
-        <v>0.1538226715525529</v>
+        <v>0.1270696463385008</v>
       </c>
       <c r="E3" t="n">
-        <v>0.1463086167939058</v>
+        <v>0.4719993135226128</v>
       </c>
       <c r="F3" t="n">
-        <v>0.03911935316019685</v>
+        <v>0.03507882890587369</v>
       </c>
       <c r="G3" t="n">
-        <v>0.0001131114249558115</v>
+        <v>8.39819750277942e-05</v>
       </c>
       <c r="H3" t="n">
-        <v>4.188787089565084e-05</v>
+        <v>3.064375249387723e-05</v>
       </c>
       <c r="I3" t="n">
-        <v>0.2776586487036053</v>
+        <v>0.2645339858650498</v>
       </c>
       <c r="J3" t="n">
-        <v>0.00129943455273878</v>
+        <v>0.0009898048859958415</v>
       </c>
       <c r="K3" t="n">
-        <v>0.0002424814918640128</v>
+        <v>0.0001780534007212298</v>
       </c>
       <c r="L3" t="n">
-        <v>0.3551602466650188</v>
+        <v>0.360748435705516</v>
       </c>
       <c r="M3" t="n">
-        <v>0.0003029620571026837</v>
+        <v>0.0002445223371025887</v>
       </c>
       <c r="N3" t="n">
-        <v>0.0004332008143224547</v>
+        <v>0.0003587012764848956</v>
       </c>
       <c r="O3" t="n">
-        <v>0.1134657253531623</v>
+        <v>0.1069056011518445</v>
       </c>
       <c r="P3" t="n">
-        <v>4.988326612235831e-07</v>
+        <v>2.578370380958563e-07</v>
       </c>
       <c r="Q3" t="n">
-        <v>2.081493896373666e-05</v>
+        <v>1.357422912321707e-05</v>
       </c>
       <c r="R3" t="n">
-        <v>0.1406218077664539</v>
+        <v>0.1352078138523419</v>
       </c>
       <c r="S3" t="n">
-        <v>0.03894652166843397</v>
+        <v>0.03694990796866792</v>
       </c>
     </row>
     <row r="4">
@@ -649,58 +649,58 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>0.005778123050014108</v>
+        <v>0.006773669736774259</v>
       </c>
       <c r="C4" t="n">
-        <v>0.1538226715525529</v>
+        <v>0.1270696463385008</v>
       </c>
       <c r="D4" t="n">
         <v>0</v>
       </c>
       <c r="E4" t="n">
-        <v>0.135156680107336</v>
+        <v>0.1279000725784861</v>
       </c>
       <c r="F4" t="n">
-        <v>0.3635398807880175</v>
+        <v>0.3825680738669138</v>
       </c>
       <c r="G4" t="n">
-        <v>0.7269427207005753</v>
+        <v>0.7691362915879639</v>
       </c>
       <c r="H4" t="n">
-        <v>0.6864117784468264</v>
+        <v>0.7271684257548012</v>
       </c>
       <c r="I4" t="n">
-        <v>0.9821542743828513</v>
+        <v>0.9975816607649222</v>
       </c>
       <c r="J4" t="n">
-        <v>0.5126501090371905</v>
+        <v>0.5525145278845934</v>
       </c>
       <c r="K4" t="n">
-        <v>0.6962304817391918</v>
+        <v>0.7417440125932547</v>
       </c>
       <c r="L4" t="n">
-        <v>0.3455688253016082</v>
+        <v>0.3505856860452268</v>
       </c>
       <c r="M4" t="n">
-        <v>0.9291968774309979</v>
+        <v>0.9632447468668599</v>
       </c>
       <c r="N4" t="n">
-        <v>0.7449007714956022</v>
+        <v>0.7739527280548124</v>
       </c>
       <c r="O4" t="n">
-        <v>0.7247788628002759</v>
+        <v>0.7064828346148219</v>
       </c>
       <c r="P4" t="n">
-        <v>0.5529411304218828</v>
+        <v>0.6160868560814229</v>
       </c>
       <c r="Q4" t="n">
-        <v>0.8043363713237719</v>
+        <v>0.8609529728696395</v>
       </c>
       <c r="R4" t="n">
-        <v>0.08432292941485321</v>
+        <v>0.08700800448111577</v>
       </c>
       <c r="S4" t="n">
-        <v>0.0820964716472162</v>
+        <v>0.08476977616474693</v>
       </c>
     </row>
     <row r="5">
@@ -710,58 +710,58 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>0.5782882316827663</v>
+        <v>0.08654873591454997</v>
       </c>
       <c r="C5" t="n">
-        <v>0.1463086167939058</v>
+        <v>0.4719993135226128</v>
       </c>
       <c r="D5" t="n">
-        <v>0.135156680107336</v>
+        <v>0.1279000725784861</v>
       </c>
       <c r="E5" t="n">
         <v>0</v>
       </c>
       <c r="F5" t="n">
-        <v>0.1707360013795562</v>
+        <v>0.001618945689942677</v>
       </c>
       <c r="G5" t="n">
-        <v>0.3486457095461422</v>
+        <v>1.187065406316367e-07</v>
       </c>
       <c r="H5" t="n">
-        <v>0.4187680761439816</v>
+        <v>6.245490078469383e-09</v>
       </c>
       <c r="I5" t="n">
-        <v>0.4915417254749917</v>
+        <v>0.2850994636229935</v>
       </c>
       <c r="J5" t="n">
-        <v>0.645318915291996</v>
+        <v>2.029546311287184e-08</v>
       </c>
       <c r="K5" t="n">
-        <v>0.6662510933640741</v>
+        <v>3.29976181900122e-09</v>
       </c>
       <c r="L5" t="n">
-        <v>0.869640100329692</v>
+        <v>0.9420070471539937</v>
       </c>
       <c r="M5" t="n">
-        <v>0.276296647921836</v>
+        <v>3.102186797595753e-05</v>
       </c>
       <c r="N5" t="n">
-        <v>0.3555239520848304</v>
+        <v>9.446537312946037e-06</v>
       </c>
       <c r="O5" t="n">
-        <v>0.4823794658847196</v>
+        <v>0.2213694445367216</v>
       </c>
       <c r="P5" t="n">
-        <v>0.3769879163640471</v>
+        <v>7.018665227729558e-17</v>
       </c>
       <c r="Q5" t="n">
-        <v>0.5734409043907681</v>
+        <v>1.854858359869705e-10</v>
       </c>
       <c r="R5" t="n">
-        <v>0.05624143293917937</v>
+        <v>2.909079053099743e-12</v>
       </c>
       <c r="S5" t="n">
-        <v>0.07955818469035211</v>
+        <v>3.506297012662958e-10</v>
       </c>
     </row>
     <row r="6">
@@ -771,58 +771,58 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>0.000937594313159404</v>
+        <v>0.0008556422323483821</v>
       </c>
       <c r="C6" t="n">
-        <v>0.03911935316019685</v>
+        <v>0.03507882890587369</v>
       </c>
       <c r="D6" t="n">
-        <v>0.3635398807880175</v>
+        <v>0.3825680738669138</v>
       </c>
       <c r="E6" t="n">
-        <v>0.1707360013795562</v>
+        <v>0.001618945689942677</v>
       </c>
       <c r="F6" t="n">
         <v>0</v>
       </c>
       <c r="G6" t="n">
-        <v>1.974872288481801e-16</v>
+        <v>2.399714176189391e-16</v>
       </c>
       <c r="H6" t="n">
-        <v>0.08604670289178744</v>
+        <v>0.09043287353072277</v>
       </c>
       <c r="I6" t="n">
-        <v>7.75470612052179e-95</v>
+        <v>1.176719245689289e-94</v>
       </c>
       <c r="J6" t="n">
-        <v>6.88725928001692e-19</v>
+        <v>8.591743183118332e-19</v>
       </c>
       <c r="K6" t="n">
-        <v>1.731040346766832e-08</v>
+        <v>1.999921545044561e-08</v>
       </c>
       <c r="L6" t="n">
-        <v>3.408706264673743e-31</v>
+        <v>3.819570820936266e-31</v>
       </c>
       <c r="M6" t="n">
-        <v>2.299093808974822e-10</v>
+        <v>2.605705997388753e-10</v>
       </c>
       <c r="N6" t="n">
-        <v>0.09723546218961994</v>
+        <v>0.09395560626429403</v>
       </c>
       <c r="O6" t="n">
-        <v>7.091842772545056e-66</v>
+        <v>9.641816352209342e-66</v>
       </c>
       <c r="P6" t="n">
-        <v>6.811783188660877e-11</v>
+        <v>8.410245630040203e-11</v>
       </c>
       <c r="Q6" t="n">
-        <v>0.004687235307140594</v>
+        <v>0.005138203659435578</v>
       </c>
       <c r="R6" t="n">
-        <v>3.790809446299059e-46</v>
+        <v>4.592263975465289e-46</v>
       </c>
       <c r="S6" t="n">
-        <v>7.534093624471843e-58</v>
+        <v>9.487615231738427e-58</v>
       </c>
     </row>
     <row r="7">
@@ -832,58 +832,58 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>6.369010827378881e-10</v>
+        <v>4.827751365533865e-10</v>
       </c>
       <c r="C7" t="n">
-        <v>0.0001131114249558115</v>
+        <v>8.39819750277942e-05</v>
       </c>
       <c r="D7" t="n">
-        <v>0.7269427207005753</v>
+        <v>0.7691362915879639</v>
       </c>
       <c r="E7" t="n">
-        <v>0.3486457095461422</v>
+        <v>1.187065406316367e-07</v>
       </c>
       <c r="F7" t="n">
-        <v>1.974872288481801e-16</v>
+        <v>2.399714176189391e-16</v>
       </c>
       <c r="G7" t="n">
         <v>0</v>
       </c>
       <c r="H7" t="n">
-        <v>1.025671153812089e-301</v>
+        <v>4.528747256512241e-301</v>
       </c>
       <c r="I7" t="n">
-        <v>4.030095793667512e-60</v>
+        <v>5.376129450652832e-60</v>
       </c>
       <c r="J7" t="n">
-        <v>1.884764228827191e-179</v>
+        <v>5.554937903422891e-179</v>
       </c>
       <c r="K7" t="n">
-        <v>2.593856756027692e-172</v>
+        <v>7.436055922806072e-172</v>
       </c>
       <c r="L7" t="n">
-        <v>3.168813912280152e-05</v>
+        <v>3.269328005525288e-05</v>
       </c>
       <c r="M7" t="n">
-        <v>6.642417843663972e-303</v>
+        <v>2.204723562991744e-302</v>
       </c>
       <c r="N7" t="n">
-        <v>1.611404131329165e-157</v>
+        <v>3.371941587635778e-157</v>
       </c>
       <c r="O7" t="n">
-        <v>6.766427497830103e-61</v>
+        <v>8.917227836036485e-61</v>
       </c>
       <c r="P7" t="n">
-        <v>3.553550893586397e-77</v>
+        <v>7.446190783924565e-77</v>
       </c>
       <c r="Q7" t="n">
-        <v>1.029697250186842e-66</v>
+        <v>2.010298407006162e-66</v>
       </c>
       <c r="R7" t="n">
-        <v>0.7623189137372203</v>
+        <v>0.754067587375348</v>
       </c>
       <c r="S7" t="n">
-        <v>0.8357631594376244</v>
+        <v>0.8443633771462299</v>
       </c>
     </row>
     <row r="8">
@@ -893,58 +893,58 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>4.335244092533622e-10</v>
+        <v>3.290047200228263e-10</v>
       </c>
       <c r="C8" t="n">
-        <v>4.188787089565084e-05</v>
+        <v>3.064375249387723e-05</v>
       </c>
       <c r="D8" t="n">
-        <v>0.6864117784468264</v>
+        <v>0.7271684257548012</v>
       </c>
       <c r="E8" t="n">
-        <v>0.4187680761439816</v>
+        <v>6.245490078469383e-09</v>
       </c>
       <c r="F8" t="n">
-        <v>0.08604670289178744</v>
+        <v>0.09043287353072277</v>
       </c>
       <c r="G8" t="n">
-        <v>1.025671153812089e-301</v>
+        <v>4.528747256512241e-301</v>
       </c>
       <c r="H8" t="n">
         <v>0</v>
       </c>
       <c r="I8" t="n">
-        <v>2.449726331083869e-10</v>
+        <v>2.727158403652608e-10</v>
       </c>
       <c r="J8" t="n">
-        <v>9.473803000416236e-149</v>
+        <v>2.465389045118758e-148</v>
       </c>
       <c r="K8" t="n">
-        <v>1.982053513222779e-179</v>
+        <v>5.777074257036877e-179</v>
       </c>
       <c r="L8" t="n">
-        <v>0.7817463702021084</v>
+        <v>0.7764225647785308</v>
       </c>
       <c r="M8" t="n">
-        <v>1.05952751000914e-201</v>
+        <v>2.73921629173763e-201</v>
       </c>
       <c r="N8" t="n">
-        <v>2.329467514240964e-253</v>
+        <v>6.151191724853308e-253</v>
       </c>
       <c r="O8" t="n">
-        <v>5.485162301238361e-13</v>
+        <v>6.162176293790057e-13</v>
       </c>
       <c r="P8" t="n">
-        <v>1.858992862382892e-89</v>
+        <v>3.958515635185607e-89</v>
       </c>
       <c r="Q8" t="n">
-        <v>5.139800015969449e-78</v>
+        <v>1.04649968419104e-77</v>
       </c>
       <c r="R8" t="n">
-        <v>0.4692335407184493</v>
+        <v>0.4626888699637891</v>
       </c>
       <c r="S8" t="n">
-        <v>0.3336112172550972</v>
+        <v>0.3281976497648921</v>
       </c>
     </row>
     <row r="9">
@@ -954,58 +954,58 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>0.01481162278016307</v>
+        <v>0.0141170298716032</v>
       </c>
       <c r="C9" t="n">
-        <v>0.2776586487036053</v>
+        <v>0.2645339858650498</v>
       </c>
       <c r="D9" t="n">
-        <v>0.9821542743828513</v>
+        <v>0.9975816607649222</v>
       </c>
       <c r="E9" t="n">
-        <v>0.4915417254749917</v>
+        <v>0.2850994636229935</v>
       </c>
       <c r="F9" t="n">
-        <v>7.75470612052179e-95</v>
+        <v>1.176719245689289e-94</v>
       </c>
       <c r="G9" t="n">
-        <v>4.030095793667512e-60</v>
+        <v>5.376129450652832e-60</v>
       </c>
       <c r="H9" t="n">
-        <v>2.449726331083869e-10</v>
+        <v>2.727158403652608e-10</v>
       </c>
       <c r="I9" t="n">
         <v>0</v>
       </c>
       <c r="J9" t="n">
-        <v>6.498222012685076e-35</v>
+        <v>8.032576831032318e-35</v>
       </c>
       <c r="K9" t="n">
-        <v>1.848364790228357e-18</v>
+        <v>2.154176888169346e-18</v>
       </c>
       <c r="L9" t="n">
-        <v>6.782179205076619e-36</v>
+        <v>7.756273311887584e-36</v>
       </c>
       <c r="M9" t="n">
-        <v>8.56384977101181e-56</v>
+        <v>1.136927004168657e-55</v>
       </c>
       <c r="N9" t="n">
-        <v>0.001911300667047139</v>
+        <v>0.00199345295230695</v>
       </c>
       <c r="O9" t="n">
-        <v>4.10626179388404e-304</v>
+        <v>1.261768075008135e-303</v>
       </c>
       <c r="P9" t="n">
-        <v>1.81205951789183e-06</v>
+        <v>2.020392298129483e-06</v>
       </c>
       <c r="Q9" t="n">
-        <v>1.98916690800386e-05</v>
+        <v>2.171757795552393e-05</v>
       </c>
       <c r="R9" t="n">
-        <v>0.4038003341097303</v>
+        <v>0.4068179789530565</v>
       </c>
       <c r="S9" t="n">
-        <v>0.005502701129368218</v>
+        <v>0.005613676122628376</v>
       </c>
     </row>
     <row r="10">
@@ -1015,28 +1015,28 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>1.859067479702329e-11</v>
+        <v>1.324049210776918e-11</v>
       </c>
       <c r="C10" t="n">
-        <v>0.00129943455273878</v>
+        <v>0.0009898048859958415</v>
       </c>
       <c r="D10" t="n">
-        <v>0.5126501090371905</v>
+        <v>0.5525145278845934</v>
       </c>
       <c r="E10" t="n">
-        <v>0.645318915291996</v>
+        <v>2.029546311287184e-08</v>
       </c>
       <c r="F10" t="n">
-        <v>6.88725928001692e-19</v>
+        <v>8.591743183118332e-19</v>
       </c>
       <c r="G10" t="n">
-        <v>1.884764228827191e-179</v>
+        <v>5.554937903422891e-179</v>
       </c>
       <c r="H10" t="n">
-        <v>9.473803000416236e-149</v>
+        <v>2.465389045118758e-148</v>
       </c>
       <c r="I10" t="n">
-        <v>6.498222012685076e-35</v>
+        <v>8.032576831032318e-35</v>
       </c>
       <c r="J10" t="n">
         <v>0</v>
@@ -1045,28 +1045,28 @@
         <v>0</v>
       </c>
       <c r="L10" t="n">
-        <v>9.504119612973177e-16</v>
+        <v>1.004197101012258e-15</v>
       </c>
       <c r="M10" t="n">
-        <v>5.102072564038504e-64</v>
+        <v>8.284482960318937e-64</v>
       </c>
       <c r="N10" t="n">
-        <v>1.319431926542275e-43</v>
+        <v>1.889597491317173e-43</v>
       </c>
       <c r="O10" t="n">
-        <v>8.975378149504911e-25</v>
+        <v>1.062825837877666e-24</v>
       </c>
       <c r="P10" t="n">
-        <v>2.457283720441464e-81</v>
+        <v>5.789304485686377e-81</v>
       </c>
       <c r="Q10" t="n">
-        <v>3.991251076704045e-60</v>
+        <v>7.992057094682185e-60</v>
       </c>
       <c r="R10" t="n">
-        <v>0.7958841424806478</v>
+        <v>0.8050515681495062</v>
       </c>
       <c r="S10" t="n">
-        <v>0.2333105763845038</v>
+        <v>0.2380095832477398</v>
       </c>
     </row>
     <row r="11">
@@ -1076,28 +1076,28 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>7.823545746664761e-11</v>
+        <v>5.65297713021527e-11</v>
       </c>
       <c r="C11" t="n">
-        <v>0.0002424814918640128</v>
+        <v>0.0001780534007212298</v>
       </c>
       <c r="D11" t="n">
-        <v>0.6962304817391918</v>
+        <v>0.7417440125932547</v>
       </c>
       <c r="E11" t="n">
-        <v>0.6662510933640741</v>
+        <v>3.29976181900122e-09</v>
       </c>
       <c r="F11" t="n">
-        <v>1.731040346766832e-08</v>
+        <v>1.999921545044561e-08</v>
       </c>
       <c r="G11" t="n">
-        <v>2.593856756027692e-172</v>
+        <v>7.436055922806072e-172</v>
       </c>
       <c r="H11" t="n">
-        <v>1.982053513222779e-179</v>
+        <v>5.777074257036877e-179</v>
       </c>
       <c r="I11" t="n">
-        <v>1.848364790228357e-18</v>
+        <v>2.154176888169346e-18</v>
       </c>
       <c r="J11" t="n">
         <v>0</v>
@@ -1106,28 +1106,28 @@
         <v>0</v>
       </c>
       <c r="L11" t="n">
-        <v>0.9377582400682594</v>
+        <v>0.9438806554439508</v>
       </c>
       <c r="M11" t="n">
-        <v>1.331916902448574e-68</v>
+        <v>2.201547128840328e-68</v>
       </c>
       <c r="N11" t="n">
-        <v>7.790551939235898e-50</v>
+        <v>1.144662810102002e-49</v>
       </c>
       <c r="O11" t="n">
-        <v>8.608425528089733e-23</v>
+        <v>1.01219226191543e-22</v>
       </c>
       <c r="P11" t="n">
-        <v>1.474028129119103e-91</v>
+        <v>3.57363727972161e-91</v>
       </c>
       <c r="Q11" t="n">
-        <v>1.112738400417991e-71</v>
+        <v>2.358682503171543e-71</v>
       </c>
       <c r="R11" t="n">
-        <v>0.6926361388704194</v>
+        <v>0.6838579896803391</v>
       </c>
       <c r="S11" t="n">
-        <v>0.446330223907014</v>
+        <v>0.4390862568941711</v>
       </c>
     </row>
     <row r="12">
@@ -1137,58 +1137,58 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>0.09315870253868073</v>
+        <v>0.09178553979175272</v>
       </c>
       <c r="C12" t="n">
-        <v>0.3551602466650188</v>
+        <v>0.360748435705516</v>
       </c>
       <c r="D12" t="n">
-        <v>0.3455688253016082</v>
+        <v>0.3505856860452268</v>
       </c>
       <c r="E12" t="n">
-        <v>0.869640100329692</v>
+        <v>0.9420070471539937</v>
       </c>
       <c r="F12" t="n">
-        <v>3.408706264673743e-31</v>
+        <v>3.819570820936266e-31</v>
       </c>
       <c r="G12" t="n">
-        <v>3.168813912280152e-05</v>
+        <v>3.269328005525288e-05</v>
       </c>
       <c r="H12" t="n">
-        <v>0.7817463702021084</v>
+        <v>0.7764225647785308</v>
       </c>
       <c r="I12" t="n">
-        <v>6.782179205076619e-36</v>
+        <v>7.756273311887584e-36</v>
       </c>
       <c r="J12" t="n">
-        <v>9.504119612973177e-16</v>
+        <v>1.004197101012258e-15</v>
       </c>
       <c r="K12" t="n">
-        <v>0.9377582400682594</v>
+        <v>0.9438806554439508</v>
       </c>
       <c r="L12" t="n">
         <v>0</v>
       </c>
       <c r="M12" t="n">
-        <v>0.3216097135098943</v>
+        <v>0.3243871017631183</v>
       </c>
       <c r="N12" t="n">
-        <v>0.6227118269479704</v>
+        <v>0.6194341515269409</v>
       </c>
       <c r="O12" t="n">
-        <v>0.004635942006977388</v>
+        <v>0.004704601898835178</v>
       </c>
       <c r="P12" t="n">
-        <v>0.8566256830427776</v>
+        <v>0.8656571852533494</v>
       </c>
       <c r="Q12" t="n">
-        <v>0.2247584828114073</v>
+        <v>0.2210494597248073</v>
       </c>
       <c r="R12" t="n">
-        <v>0.03364135531183689</v>
+        <v>0.03393081628861537</v>
       </c>
       <c r="S12" t="n">
-        <v>8.092576235101778e-11</v>
+        <v>8.445197987089489e-11</v>
       </c>
     </row>
     <row r="13">
@@ -1198,58 +1198,58 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>2.03499470752718e-06</v>
+        <v>1.74318497422886e-06</v>
       </c>
       <c r="C13" t="n">
-        <v>0.0003029620571026837</v>
+        <v>0.0002445223371025887</v>
       </c>
       <c r="D13" t="n">
-        <v>0.9291968774309979</v>
+        <v>0.9632447468668599</v>
       </c>
       <c r="E13" t="n">
-        <v>0.276296647921836</v>
+        <v>3.102186797595753e-05</v>
       </c>
       <c r="F13" t="n">
-        <v>2.299093808974822e-10</v>
+        <v>2.605705997388753e-10</v>
       </c>
       <c r="G13" t="n">
-        <v>6.642417843663972e-303</v>
+        <v>2.204723562991744e-302</v>
       </c>
       <c r="H13" t="n">
-        <v>1.05952751000914e-201</v>
+        <v>2.73921629173763e-201</v>
       </c>
       <c r="I13" t="n">
-        <v>8.56384977101181e-56</v>
+        <v>1.136927004168657e-55</v>
       </c>
       <c r="J13" t="n">
-        <v>5.102072564038504e-64</v>
+        <v>8.284482960318937e-64</v>
       </c>
       <c r="K13" t="n">
-        <v>1.331916902448574e-68</v>
+        <v>2.201547128840328e-68</v>
       </c>
       <c r="L13" t="n">
-        <v>0.3216097135098943</v>
+        <v>0.3243871017631183</v>
       </c>
       <c r="M13" t="n">
         <v>0</v>
       </c>
       <c r="N13" t="n">
-        <v>7.060115529731066e-213</v>
+        <v>1.822167940285636e-212</v>
       </c>
       <c r="O13" t="n">
-        <v>1.775595697211848e-68</v>
+        <v>2.437049086352392e-68</v>
       </c>
       <c r="P13" t="n">
-        <v>2.869250138656061e-47</v>
+        <v>4.419225991016588e-47</v>
       </c>
       <c r="Q13" t="n">
-        <v>2.567526652382389e-46</v>
+        <v>3.940820623518739e-46</v>
       </c>
       <c r="R13" t="n">
-        <v>0.5363613111752364</v>
+        <v>0.5310370474777102</v>
       </c>
       <c r="S13" t="n">
-        <v>0.635887052626617</v>
+        <v>0.6299987408681955</v>
       </c>
     </row>
     <row r="14">
@@ -1259,58 +1259,58 @@
         </is>
       </c>
       <c r="B14" t="n">
-        <v>3.437593850426097e-06</v>
+        <v>3.003624054421726e-06</v>
       </c>
       <c r="C14" t="n">
-        <v>0.0004332008143224547</v>
+        <v>0.0003587012764848956</v>
       </c>
       <c r="D14" t="n">
-        <v>0.7449007714956022</v>
+        <v>0.7739527280548124</v>
       </c>
       <c r="E14" t="n">
-        <v>0.3555239520848304</v>
+        <v>9.446537312946037e-06</v>
       </c>
       <c r="F14" t="n">
-        <v>0.09723546218961994</v>
+        <v>0.09395560626429403</v>
       </c>
       <c r="G14" t="n">
-        <v>1.611404131329165e-157</v>
+        <v>3.371941587635778e-157</v>
       </c>
       <c r="H14" t="n">
-        <v>2.329467514240964e-253</v>
+        <v>6.151191724853308e-253</v>
       </c>
       <c r="I14" t="n">
-        <v>0.001911300667047139</v>
+        <v>0.00199345295230695</v>
       </c>
       <c r="J14" t="n">
-        <v>1.319431926542275e-43</v>
+        <v>1.889597491317173e-43</v>
       </c>
       <c r="K14" t="n">
-        <v>7.790551939235898e-50</v>
+        <v>1.144662810102002e-49</v>
       </c>
       <c r="L14" t="n">
-        <v>0.6227118269479704</v>
+        <v>0.6194341515269409</v>
       </c>
       <c r="M14" t="n">
-        <v>7.060115529731066e-213</v>
+        <v>1.822167940285636e-212</v>
       </c>
       <c r="N14" t="n">
         <v>0</v>
       </c>
       <c r="O14" t="n">
-        <v>0.00024406226604551</v>
+        <v>0.0002558955928728002</v>
       </c>
       <c r="P14" t="n">
-        <v>8.110869746639962e-48</v>
+        <v>1.168204901530113e-47</v>
       </c>
       <c r="Q14" t="n">
-        <v>1.313249011983679e-46</v>
+        <v>1.923052467608921e-46</v>
       </c>
       <c r="R14" t="n">
-        <v>0.4123224833925239</v>
+        <v>0.4082589943535039</v>
       </c>
       <c r="S14" t="n">
-        <v>0.3608206198636272</v>
+        <v>0.3570283346696159</v>
       </c>
     </row>
     <row r="15">
@@ -1320,58 +1320,58 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>0.04057990178849622</v>
+        <v>0.03900395999926402</v>
       </c>
       <c r="C15" t="n">
-        <v>0.1134657253531623</v>
+        <v>0.1069056011518445</v>
       </c>
       <c r="D15" t="n">
-        <v>0.7247788628002759</v>
+        <v>0.7064828346148219</v>
       </c>
       <c r="E15" t="n">
-        <v>0.4823794658847196</v>
+        <v>0.2213694445367216</v>
       </c>
       <c r="F15" t="n">
-        <v>7.091842772545056e-66</v>
+        <v>9.641816352209342e-66</v>
       </c>
       <c r="G15" t="n">
-        <v>6.766427497830103e-61</v>
+        <v>8.917227836036485e-61</v>
       </c>
       <c r="H15" t="n">
-        <v>5.485162301238361e-13</v>
+        <v>6.162176293790057e-13</v>
       </c>
       <c r="I15" t="n">
-        <v>4.10626179388404e-304</v>
+        <v>1.261768075008135e-303</v>
       </c>
       <c r="J15" t="n">
-        <v>8.975378149504911e-25</v>
+        <v>1.062825837877666e-24</v>
       </c>
       <c r="K15" t="n">
-        <v>8.608425528089733e-23</v>
+        <v>1.01219226191543e-22</v>
       </c>
       <c r="L15" t="n">
-        <v>0.004635942006977388</v>
+        <v>0.004704601898835178</v>
       </c>
       <c r="M15" t="n">
-        <v>1.775595697211848e-68</v>
+        <v>2.437049086352392e-68</v>
       </c>
       <c r="N15" t="n">
-        <v>0.00024406226604551</v>
+        <v>0.0002558955928728002</v>
       </c>
       <c r="O15" t="n">
         <v>0</v>
       </c>
       <c r="P15" t="n">
-        <v>1.386618343411048e-07</v>
+        <v>1.545724460280185e-07</v>
       </c>
       <c r="Q15" t="n">
-        <v>1.357405845675919e-07</v>
+        <v>1.498136735883907e-07</v>
       </c>
       <c r="R15" t="n">
-        <v>0.9330764752296365</v>
+        <v>0.9368101796160265</v>
       </c>
       <c r="S15" t="n">
-        <v>0.5942571143756611</v>
+        <v>0.5977361810081139</v>
       </c>
     </row>
     <row r="16">
@@ -1381,58 +1381,58 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>4.407385311917058e-11</v>
+        <v>2.582053559427021e-11</v>
       </c>
       <c r="C16" t="n">
-        <v>4.988326612235831e-07</v>
+        <v>2.578370380958563e-07</v>
       </c>
       <c r="D16" t="n">
-        <v>0.5529411304218828</v>
+        <v>0.6160868560814229</v>
       </c>
       <c r="E16" t="n">
-        <v>0.3769879163640471</v>
+        <v>7.018665227729558e-17</v>
       </c>
       <c r="F16" t="n">
-        <v>6.811783188660877e-11</v>
+        <v>8.410245630040203e-11</v>
       </c>
       <c r="G16" t="n">
-        <v>3.553550893586397e-77</v>
+        <v>7.446190783924565e-77</v>
       </c>
       <c r="H16" t="n">
-        <v>1.858992862382892e-89</v>
+        <v>3.958515635185607e-89</v>
       </c>
       <c r="I16" t="n">
-        <v>1.81205951789183e-06</v>
+        <v>2.020392298129483e-06</v>
       </c>
       <c r="J16" t="n">
-        <v>2.457283720441464e-81</v>
+        <v>5.789304485686377e-81</v>
       </c>
       <c r="K16" t="n">
-        <v>1.474028129119103e-91</v>
+        <v>3.57363727972161e-91</v>
       </c>
       <c r="L16" t="n">
-        <v>0.8566256830427776</v>
+        <v>0.8656571852533494</v>
       </c>
       <c r="M16" t="n">
-        <v>2.869250138656061e-47</v>
+        <v>4.419225991016588e-47</v>
       </c>
       <c r="N16" t="n">
-        <v>8.110869746639962e-48</v>
+        <v>1.168204901530113e-47</v>
       </c>
       <c r="O16" t="n">
-        <v>1.386618343411048e-07</v>
+        <v>1.545724460280185e-07</v>
       </c>
       <c r="P16" t="n">
         <v>0</v>
       </c>
       <c r="Q16" t="n">
-        <v>2.095860545368796e-204</v>
+        <v>9.121771058524368e-204</v>
       </c>
       <c r="R16" t="n">
-        <v>0.006401426335289058</v>
+        <v>0.006690001764821096</v>
       </c>
       <c r="S16" t="n">
-        <v>0.002548964116787642</v>
+        <v>0.00267375908048787</v>
       </c>
     </row>
     <row r="17">
@@ -1442,58 +1442,58 @@
         </is>
       </c>
       <c r="B17" t="n">
-        <v>3.71175767927445e-10</v>
+        <v>2.543843960175141e-10</v>
       </c>
       <c r="C17" t="n">
-        <v>2.081493896373666e-05</v>
+        <v>1.357422912321707e-05</v>
       </c>
       <c r="D17" t="n">
-        <v>0.8043363713237719</v>
+        <v>0.8609529728696395</v>
       </c>
       <c r="E17" t="n">
-        <v>0.5734409043907681</v>
+        <v>1.854858359869705e-10</v>
       </c>
       <c r="F17" t="n">
-        <v>0.004687235307140594</v>
+        <v>0.005138203659435578</v>
       </c>
       <c r="G17" t="n">
-        <v>1.029697250186842e-66</v>
+        <v>2.010298407006162e-66</v>
       </c>
       <c r="H17" t="n">
-        <v>5.139800015969449e-78</v>
+        <v>1.04649968419104e-77</v>
       </c>
       <c r="I17" t="n">
-        <v>1.98916690800386e-05</v>
+        <v>2.171757795552393e-05</v>
       </c>
       <c r="J17" t="n">
-        <v>3.991251076704045e-60</v>
+        <v>7.992057094682185e-60</v>
       </c>
       <c r="K17" t="n">
-        <v>1.112738400417991e-71</v>
+        <v>2.358682503171543e-71</v>
       </c>
       <c r="L17" t="n">
-        <v>0.2247584828114073</v>
+        <v>0.2210494597248073</v>
       </c>
       <c r="M17" t="n">
-        <v>2.567526652382389e-46</v>
+        <v>3.940820623518739e-46</v>
       </c>
       <c r="N17" t="n">
-        <v>1.313249011983679e-46</v>
+        <v>1.923052467608921e-46</v>
       </c>
       <c r="O17" t="n">
-        <v>1.357405845675919e-07</v>
+        <v>1.498136735883907e-07</v>
       </c>
       <c r="P17" t="n">
-        <v>2.095860545368796e-204</v>
+        <v>9.121771058524368e-204</v>
       </c>
       <c r="Q17" t="n">
         <v>0</v>
       </c>
       <c r="R17" t="n">
-        <v>0.002269131730379557</v>
+        <v>0.002151996851687472</v>
       </c>
       <c r="S17" t="n">
-        <v>0.01288823543733667</v>
+        <v>0.01232890870192866</v>
       </c>
     </row>
     <row r="18">
@@ -1503,58 +1503,58 @@
         </is>
       </c>
       <c r="B18" t="n">
-        <v>0.6702671245435687</v>
+        <v>0.6623627930669869</v>
       </c>
       <c r="C18" t="n">
-        <v>0.1406218077664539</v>
+        <v>0.1352078138523419</v>
       </c>
       <c r="D18" t="n">
-        <v>0.08432292941485321</v>
+        <v>0.08700800448111577</v>
       </c>
       <c r="E18" t="n">
-        <v>0.05624143293917937</v>
+        <v>2.909079053099743e-12</v>
       </c>
       <c r="F18" t="n">
-        <v>3.790809446299059e-46</v>
+        <v>4.592263975465289e-46</v>
       </c>
       <c r="G18" t="n">
-        <v>0.7623189137372203</v>
+        <v>0.754067587375348</v>
       </c>
       <c r="H18" t="n">
-        <v>0.4692335407184493</v>
+        <v>0.4626888699637891</v>
       </c>
       <c r="I18" t="n">
-        <v>0.4038003341097303</v>
+        <v>0.4068179789530565</v>
       </c>
       <c r="J18" t="n">
-        <v>0.7958841424806478</v>
+        <v>0.8050515681495062</v>
       </c>
       <c r="K18" t="n">
-        <v>0.6926361388704194</v>
+        <v>0.6838579896803391</v>
       </c>
       <c r="L18" t="n">
-        <v>0.03364135531183689</v>
+        <v>0.03393081628861537</v>
       </c>
       <c r="M18" t="n">
-        <v>0.5363613111752364</v>
+        <v>0.5310370474777102</v>
       </c>
       <c r="N18" t="n">
-        <v>0.4123224833925239</v>
+        <v>0.4082589943535039</v>
       </c>
       <c r="O18" t="n">
-        <v>0.9330764752296365</v>
+        <v>0.9368101796160265</v>
       </c>
       <c r="P18" t="n">
-        <v>0.006401426335289058</v>
+        <v>0.006690001764821096</v>
       </c>
       <c r="Q18" t="n">
-        <v>0.002269131730379557</v>
+        <v>0.002151996851687472</v>
       </c>
       <c r="R18" t="n">
         <v>0</v>
       </c>
       <c r="S18" t="n">
-        <v>3.931863341420891e-318</v>
+        <v>1.207141699302293e-317</v>
       </c>
     </row>
     <row r="19">
@@ -1564,55 +1564,55 @@
         </is>
       </c>
       <c r="B19" t="n">
-        <v>0.5169353273419229</v>
+        <v>0.5098068507681475</v>
       </c>
       <c r="C19" t="n">
-        <v>0.03894652166843397</v>
+        <v>0.03694990796866792</v>
       </c>
       <c r="D19" t="n">
-        <v>0.0820964716472162</v>
+        <v>0.08476977616474693</v>
       </c>
       <c r="E19" t="n">
-        <v>0.07955818469035211</v>
+        <v>3.506297012662958e-10</v>
       </c>
       <c r="F19" t="n">
-        <v>7.534093624471843e-58</v>
+        <v>9.487615231738427e-58</v>
       </c>
       <c r="G19" t="n">
-        <v>0.8357631594376244</v>
+        <v>0.8443633771462299</v>
       </c>
       <c r="H19" t="n">
-        <v>0.3336112172550972</v>
+        <v>0.3281976497648921</v>
       </c>
       <c r="I19" t="n">
-        <v>0.005502701129368218</v>
+        <v>0.005613676122628376</v>
       </c>
       <c r="J19" t="n">
-        <v>0.2333105763845038</v>
+        <v>0.2380095832477398</v>
       </c>
       <c r="K19" t="n">
-        <v>0.446330223907014</v>
+        <v>0.4390862568941711</v>
       </c>
       <c r="L19" t="n">
-        <v>8.092576235101778e-11</v>
+        <v>8.445197987089489e-11</v>
       </c>
       <c r="M19" t="n">
-        <v>0.635887052626617</v>
+        <v>0.6299987408681955</v>
       </c>
       <c r="N19" t="n">
-        <v>0.3608206198636272</v>
+        <v>0.3570283346696159</v>
       </c>
       <c r="O19" t="n">
-        <v>0.5942571143756611</v>
+        <v>0.5977361810081139</v>
       </c>
       <c r="P19" t="n">
-        <v>0.002548964116787642</v>
+        <v>0.00267375908048787</v>
       </c>
       <c r="Q19" t="n">
-        <v>0.01288823543733667</v>
+        <v>0.01232890870192866</v>
       </c>
       <c r="R19" t="n">
-        <v>3.931863341420891e-318</v>
+        <v>1.207141699302293e-317</v>
       </c>
       <c r="S19" t="n">
         <v>0</v>

</xml_diff>